<commit_message>
Strip images from Set up Report sheet in template
</commit_message>
<xml_diff>
--- a/data/static/report_template.xlsx
+++ b/data/static/report_template.xlsx
@@ -3733,249 +3733,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>71200</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>101923</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>295865</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>314618</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1" descr="A picture containing dark, laptop, sitting, lit&#10;&#10;Description automatically generated">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E567DBCB-955D-264A-945C-3F7DE7571DA9}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2408000" y="7963223"/>
-          <a:ext cx="224665" cy="212695"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="bg1"/>
-        </a:solidFill>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>57490</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>100004</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>321468</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>326579</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2" descr="A picture containing dark, black, white, sitting&#10;&#10;Description automatically generated">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9B425DB1-FAD4-E74F-83F1-73CBEC2876F1}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2394290" y="8342304"/>
-          <a:ext cx="263978" cy="226575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="bg1"/>
-        </a:solidFill>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
-      <xdr:row>55</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>4965246</xdr:colOff>
-      <xdr:row>55</xdr:row>
-      <xdr:rowOff>3263900</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F8339857-9163-2047-A97B-F91669EB5903}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="14300200" y="15151100"/>
-          <a:ext cx="4889046" cy="3263900"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2286000</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>12700</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>363099</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>6350</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{24B968A4-3818-5B4A-86BF-A680BCAFAB3B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2286000" y="7493000"/>
-          <a:ext cx="413899" cy="374650"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>115972</xdr:colOff>
-      <xdr:row>57</xdr:row>
-      <xdr:rowOff>101600</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>4893382</xdr:colOff>
-      <xdr:row>57</xdr:row>
-      <xdr:rowOff>1625600</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{484DE4FF-4FAE-EA44-9098-DC7F749FDDD6}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="14339972" y="18745200"/>
-          <a:ext cx="4777410" cy="1524000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>